<commit_message>
chore: update schedules 2026-10-11
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -570,17 +570,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>06-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1595,32 +1595,32 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>00642</t>
+          <t>00442</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>13-Oct-2026</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>29</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>06-Oct-2026</t>
+          <t>13-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,32 +1699,32 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>00441</t>
+          <t>00643</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>11-Oct-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1771,12 +1771,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,32 +1803,32 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>00442</t>
+          <t>00644</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>13-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>13-Oct-2026</t>
+          <t>18-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>00643</t>
+          <t>01200</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1892,47 +1892,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>18-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>01200</t>
+          <t>01201</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>01201</t>
+          <t>01202</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,47 +2100,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>30-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>01204</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>22-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>ESL TBN1</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>02647</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>19-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>01202</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>19-Nov-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2323,12 +2323,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2338,17 +2338,17 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-10 05:02 UTC</t>
+          <t>2026-10-11 04:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2442,17 +2442,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,47 +2568,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>12-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>01095</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>10-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2620,47 +2620,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>01095</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-10 05:03 UTC</t>
+          <t>2026-10-11 04:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-12
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>25-Nov-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>19-Dec-2026</t>
+          <t>16-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>06-Jan-2027</t>
+          <t>02-Jan-2027</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-11 04:51 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
+          <t>09-Oct-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>YOU SHUN JI 008</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>01065</t>
+          <t>2639E</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>YOU SHUN JI 008</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2639E</t>
+          <t>01066</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>11-Oct-2026</t>
+          <t>12-Oct-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>01066</t>
+          <t>01095</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,47 +2568,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>01095</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>25-Nov-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2620,47 +2620,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>01067</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>10-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>01067</t>
+          <t>01096</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>01068</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>01097</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01069</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-11 04:52 UTC</t>
+          <t>2026-10-12 05:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-13
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>21-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -575,12 +575,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -726,17 +726,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -783,12 +783,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>25-Nov-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -909,22 +909,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>08-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -961,22 +961,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,17 +1013,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>10-Dec-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>30-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,17 +1065,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>30-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16-Dec-2026</t>
+          <t>29-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>02-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-12 05:05 UTC</t>
+          <t>2026-10-13 06:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>21-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>12-Oct-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1595,32 +1595,32 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>00442</t>
+          <t>00643</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>13-Oct-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1632,12 +1632,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>13-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>00643</t>
+          <t>00644</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1736,47 +1736,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>00442</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1788,47 +1788,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>21-Oct-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>18-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>01200</t>
+          <t>00645</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,17 +1922,17 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,42 +2053,42 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>00443</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>BUSAN</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
           <t>26-Oct-2026</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>01202</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>NINGBO</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>15-Nov-2026</t>
-        </is>
-      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,47 +2100,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>19-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>01202</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>30-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>01204</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>01-Dec-2026</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>ESL KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>02648</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>19-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2323,12 +2323,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2338,34 +2338,34 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2375,64 +2375,64 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>YOU SHUN JI 008</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2639E</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>11-Oct-2026</t>
+          <t>09-Oct-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>YOU SHUN JI 008</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>01066</t>
+          <t>2639E</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2516,47 +2516,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>01095</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,47 +2568,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>01066</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>07-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>25-Nov-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>12-Oct-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>01067</t>
+          <t>01095</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2672,47 +2672,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>01067</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01096</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-12 05:06 UTC</t>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -2833,42 +2833,146 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
+          <t>19-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>01068</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-10-13 06:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>20-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>01097</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>28-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-10-13 06:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
           <t>23-Oct-2026</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>FEEDER</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>01069</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>31-Oct-2026</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
-        <is>
-          <t>2026-10-12 05:06 UTC</t>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-10-13 06:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-14
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -753,22 +753,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -778,17 +778,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -805,22 +805,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -882,17 +882,17 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -919,12 +919,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -961,22 +961,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,22 +1013,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10-Dec-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>30-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,17 +1065,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>30-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>29-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1152,39 +1152,39 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-13 06:05 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>29-Dec-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1194,17 +1194,17 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1350,17 +1350,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>20-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1402,17 +1402,17 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1454,17 +1454,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>08-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1506,17 +1506,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>30-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>08-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1558,69 +1558,69 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>30-Dec-2026</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>00643</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:08 UTC</t>
         </is>
       </c>
     </row>
@@ -1632,47 +1632,47 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>12-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CHANGHENG27</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>00643</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>22-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>BHUDTHI BHUM</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>026E6</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1684,47 +1684,47 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1751,32 +1751,32 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>00442</t>
+          <t>00644</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1788,47 +1788,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>16-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>00442</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>21-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>PHOEBE</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>026E7</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1840,47 +1840,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>21-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1892,47 +1892,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>20-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>CHANGHENG26</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>06083</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>29-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>KMTC DOHA</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>02643</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1944,37 +1944,37 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>01201</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1996,47 +1996,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>22-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CHANGHENG27</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>00645</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>22-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>ESL TBN1</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>02647</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2048,47 +2048,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,47 +2100,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>00443</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>04-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>02645</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2152,47 +2152,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>01202</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2209,42 +2209,42 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
+          <t>26-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>HUAXIN968</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>00646</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>NINGBO</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>30-Oct-2026</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>01204</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>NINGBO</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>19-Nov-2026</t>
-        </is>
-      </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,37 +2256,37 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>26-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>01202</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>01-Dec-2026</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>ESL KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>02648</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2360,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2412,64 +2412,64 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>30-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>01204</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>27-Dec-2026</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>02652</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>19-Nov-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2479,64 +2479,64 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>YOU SHUN JI 008</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2639E</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2546,17 +2546,17 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2620,47 +2620,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>01095</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2672,47 +2672,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>12-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>01095</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>13-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2724,47 +2724,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01067</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>01067</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>01096</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01068</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-13 06:06 UTC</t>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2937,42 +2937,198 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>20-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>01097</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>28-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:09 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>13-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ECMX</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>KMTC LONG BEACH</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>02644</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>01-Dec-2026</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:09 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
           <t>23-Oct-2026</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>FEEDER</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>01069</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>31-Oct-2026</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2026-10-13 06:06 UTC</t>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:09 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>24-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>01098</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>01-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:09 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-15
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,22 +493,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>21-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>026E5</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>21-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,17 +570,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -622,17 +622,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -649,22 +649,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -674,17 +674,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -711,12 +711,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -763,12 +763,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -778,17 +778,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -805,22 +805,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>08-Dec-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -882,17 +882,17 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>02-Dec-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -919,12 +919,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>21-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -961,22 +961,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,22 +1013,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>30-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1117,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>12-Jan-2027</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1350,17 +1350,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1402,17 +1402,17 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>20-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1454,17 +1454,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>21-Dec-2026</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>10-Dec-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1506,17 +1506,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>08-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>30-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1595,12 +1595,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>12-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-14 04:08 UTC</t>
+          <t>2026-10-15 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1818,17 +1818,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>21-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1944,47 +1944,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>22-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CHANGHENG27</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>00645</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>25-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>PHOEBE</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>026E7</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1996,47 +1996,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2048,47 +2048,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>00443</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,47 +2100,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2152,47 +2152,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>00646</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,37 +2256,37 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>26-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>01202</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>09-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>02645</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>01202</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2360,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>30-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>01204</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>22-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>ESL TBN1</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>02647</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>19-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2432,7 +2432,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>19-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2464,99 +2464,99 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>02-Dec-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>21-Dec-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>01066</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,47 +2568,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>01066</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2620,47 +2620,47 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>12-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>01095</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>19-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>ESL BUSAN</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>02642</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2672,47 +2672,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>01095</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2724,47 +2724,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>01067</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>27-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>ESL SHEKOU</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>026D7</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01067</t>
+          <t>01096</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>01068</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>01097</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2932,47 +2932,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2984,47 +2984,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>01069</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>13-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>01098</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3076,59 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-14 04:09 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>24-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>01098</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>01-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-10-14 04:09 UTC</t>
+          <t>2026-10-15 03:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-16
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,22 +493,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>21-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,17 +570,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -649,22 +649,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -674,17 +674,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -701,22 +701,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -726,17 +726,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -753,22 +753,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -778,17 +778,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -815,12 +815,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>08-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -909,22 +909,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>02-Dec-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>21-Dec-2026</t>
+          <t>08-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -961,22 +961,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -986,17 +986,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,17 +1013,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12-Dec-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>12-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1283,12 +1283,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1350,17 +1350,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>20-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1402,17 +1402,17 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1454,17 +1454,17 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>21-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10-Dec-2026</t>
+          <t>28-Nov-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>10-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1543,12 +1543,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1595,12 +1595,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>12-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-15 03:51 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1944,47 +1944,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1996,47 +1996,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>22-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CHANGHENG27</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>00645</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>29-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>KMTC DOHA</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>02643</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2048,47 +2048,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,47 +2100,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>00443</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>04-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>02645</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2152,47 +2152,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>26-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>HUAXIN968</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>00646</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>09-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>02645</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2256,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>01202</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>01204</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>19-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>02-Dec-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2494,34 +2494,34 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>21-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>11-Oct-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2536,59 +2536,59 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>01066</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2598,17 +2598,17 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>21-Oct-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2687,12 +2687,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2702,17 +2702,17 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2776,47 +2776,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>01096</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01068</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2932,47 +2932,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>20-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>01097</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>13-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2984,47 +2984,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-15 03:52 UTC</t>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>
@@ -3041,42 +3041,146 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>01069</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-10-16 03:47 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
           <t>24-Oct-2026</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>FEEDER</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>01098</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>01-Nov-2026</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-10-15 03:52 UTC</t>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-10-16 03:47 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>01070</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>04-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-10-16 03:47 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-17
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -810,17 +810,17 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -882,17 +882,17 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-16 03:46 UTC</t>
+          <t>2026-10-17 03:36 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>18-Oct-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>20-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>28-Nov-2026</t>
+          <t>27-Nov-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1511,12 +1511,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10-Dec-2026</t>
+          <t>09-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>00643</t>
+          <t>00644</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1662,17 +1662,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1751,32 +1751,32 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>00442</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1788,47 +1788,47 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>00442</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1840,47 +1840,47 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>CHANGHENG26</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>06083</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1892,47 +1892,47 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>06083</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1944,47 +1944,47 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>22-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CHANGHENG27</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>00645</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>25-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>PHOEBE</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>026E7</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -1996,47 +1996,47 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2048,47 +2048,47 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>00443</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,47 +2100,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2152,47 +2152,47 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>00646</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2256,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2323,32 +2323,32 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>02-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2412,47 +2412,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2464,37 +2464,37 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>07-Dec-2026</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>01206</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>30-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>ESL KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>02648</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2516,47 +2516,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,99 +2568,99 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>11-Dec-2026</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>01207</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>27-Dec-2026</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>02652</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>12-Oct-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>01095</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2672,47 +2672,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>15-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>01067</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>21-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>ESL BUSAN</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>02642</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2724,47 +2724,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01067</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2776,47 +2776,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>16-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>01096</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>27-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>ESL SHEKOU</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>026D7</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>01068</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>01097</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2932,47 +2932,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -2984,47 +2984,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>01069</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>13-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>01098</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>01070</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>01070</t>
+          <t>01099</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-16 03:47 UTC</t>
+          <t>2026-10-17 03:37 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-18
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>14-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-17 03:36 UTC</t>
+          <t>2026-10-18 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27-Nov-2026</t>
+          <t>28-Nov-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1511,12 +1511,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1927,12 +1927,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-17 03:37 UTC</t>
+          <t>2026-10-18 03:44 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-19
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-18 03:43 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>18-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1407,12 +1407,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1647,32 +1647,32 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>00442</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,32 +1751,32 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>00442</t>
+          <t>00644</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1788,12 +1788,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,17 +1818,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2135,12 +2135,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-18 03:44 UTC</t>
+          <t>2026-10-19 03:54 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-20
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -659,32 +659,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -701,22 +701,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -726,17 +726,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -763,32 +763,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>28-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>31</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -805,22 +805,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -882,17 +882,17 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -909,42 +909,42 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>08-Dec-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -961,22 +961,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -986,17 +986,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,22 +1013,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1038,17 +1038,17 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12-Dec-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1075,32 +1075,32 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1117,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>14-Dec-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>08-Dec-2026</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -1169,22 +1169,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>29-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1194,34 +1194,34 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1231,22 +1231,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1256,39 +1256,39 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1298,34 +1298,34 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1350,34 +1350,34 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1387,49 +1387,49 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>14-Dec-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1454,34 +1454,34 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>28-Nov-2026</t>
+          <t>14-Dec-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1491,49 +1491,49 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>09-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>09-Dec-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1543,64 +1543,64 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>16-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNNGB→AEJEA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>12-Dec-2026</t>
+          <t>29-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1610,86 +1610,86 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-19 03:53 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>00442</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,86 +1714,86 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,86 +1818,86 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>06083</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>27-Nov-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,86 +1922,86 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>10-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,17 +2026,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>00442</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2078,17 +2078,17 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2130,17 +2130,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>00644</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>21-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2234,17 +2234,17 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2271,32 +2271,32 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>CHANGHENG26</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>06083</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>02-Nov-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2375,12 +2375,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>00645</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2390,17 +2390,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2427,12 +2427,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2479,32 +2479,32 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>00443</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2516,12 +2516,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2546,17 +2546,17 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>01207</t>
+          <t>00646</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2598,17 +2598,17 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2650,34 +2650,34 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2687,101 +2687,101 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>01067</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2796,96 +2796,96 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2900,59 +2900,59 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2962,34 +2962,34 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3004,79 +3004,79 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>01207</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:05 UTC</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>16-Oct-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>01070</t>
+          <t>01096</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-19 03:54 UTC</t>
+          <t>2026-10-20 04:06 UTC</t>
         </is>
       </c>
     </row>
@@ -3140,47 +3140,463 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ECMX</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ESL SHEKOU</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>026D7</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>22-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>WUHAN</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>19-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>01068</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>20-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>01097</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
         <is>
           <t>28-Oct-2026</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>13-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ECMX</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>KMTC LONG BEACH</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>02644</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>01-Dec-2026</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
         <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>FEEDER</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>01069</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>24-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>01098</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>01-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ZHONG YI RUN HAI</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2642E</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>04-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>28-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
         <is>
           <t>01099</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H60" t="inlineStr">
         <is>
           <t>05-Nov-2026</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-10-19 03:54 UTC</t>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>01071</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>08-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>2026-10-20 04:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-21
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,22 +493,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -545,22 +545,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,17 +570,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -617,22 +617,22 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -659,32 +659,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>17-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -721,22 +721,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -753,42 +753,42 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>28-Nov-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -805,22 +805,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -877,22 +877,22 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -909,42 +909,42 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -961,22 +961,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -986,17 +986,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1033,22 +1033,22 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,42 +1065,42 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>22-Nov-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>08-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1117,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>08-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1189,22 +1189,22 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,42 +1221,42 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>25-Dec-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,17 +1273,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1298,17 +1298,17 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>02-Jan-2027</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1345,22 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>05-Jan-2027</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>17-Dec-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1387,32 +1387,32 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14-Dec-2026</t>
+          <t>17-Dec-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,32 +1439,32 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>11-Jan-2027</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,42 +1481,42 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>14-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>09-Jan-2027</t>
+          <t>15-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1543,32 +1543,32 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>16-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,42 +1585,42 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>29-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>22-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1766,17 +1766,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>27-Nov-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>27-Nov-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,17 +1922,17 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>02-Jan-2027</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1974,17 +1974,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>12-Dec-2026</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2063,17 +2063,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00442</t>
+          <t>00644</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2083,12 +2083,12 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,12 +2100,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2130,17 +2130,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2167,12 +2167,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>CHANGHENG26</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>06083</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>21-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>22-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>CHANGHENG27</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>00645</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>23-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>BHUDTHI BHUM</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>026E6</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2256,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>06083</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>00443</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>BUSAN</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
           <t>26-Oct-2026</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>PHOEBE</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>026E7</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>14-Nov-2026</t>
-        </is>
-      </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2360,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2412,47 +2412,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>26-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>HUAXIN968</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>00646</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>29-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>KMTC DOHA</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>02643</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2516,47 +2516,47 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2598,17 +2598,17 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2635,12 +2635,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2650,17 +2650,17 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2687,32 +2687,32 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2724,47 +2724,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2781,7 +2781,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2843,12 +2843,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>01207</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2947,12 +2947,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2972,24 +2972,24 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3004,59 +3004,59 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>01207</t>
+          <t>01068</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3066,17 +3066,17 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-20 04:05 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>01096</t>
+          <t>01097</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3140,47 +3140,47 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>01069</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>27-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>ESL SHEKOU</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>026D7</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3192,47 +3192,47 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3249,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01098</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3296,47 +3296,47 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ZHONG YI RUN HAI</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2642E</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>13-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>01099</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3405,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>01071</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3467,12 +3467,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ZHONG YI RUN HAI</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2642E</t>
+          <t>01200</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3492,111 +3492,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-10-20 04:06 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>28-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>01099</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>05-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>2026-10-20 04:06 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>31-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>01071</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>08-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>2026-10-20 04:06 UTC</t>
+          <t>2026-10-21 03:55 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-22
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>17-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1147,12 +1147,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>14-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>02-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>14-Dec-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>05-Jan-2027</t>
+          <t>06-Jan-2027</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -1630,118 +1630,90 @@
           <t>CNTAO→AEJEA</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>QINGDAO</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>24-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>026E7</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>14-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
+          <t>(No schedule found)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>CHANGHENG26</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>06083</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,12 +1723,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1766,138 +1738,138 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>00645</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>27-Nov-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>00443</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1879,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,7 +1894,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>02-Jan-2027</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1932,76 +1904,76 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>00646</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>25-Dec-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2016,7 +1988,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,17 +1998,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2025,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2063,12 +2035,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>DINGSHENG7</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00644</t>
+          <t>06068</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2078,17 +2050,17 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2100,47 +2072,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2129,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2167,12 +2139,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>06083</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2182,17 +2154,17 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2176,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2228,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2280,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2332,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2412,47 +2384,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2464,47 +2436,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>01207</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2516,64 +2488,64 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>19-Oct-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2588,59 +2560,59 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>01068</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2650,34 +2622,34 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2687,205 +2659,205 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>01097</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>01069</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>01098</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2895,84 +2867,84 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ZHONG YI RUN HAI</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01207</t>
+          <t>2642E</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>01099</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-21 03:54 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2961,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3004,7 +2976,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>01071</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3014,7 +2986,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3024,7 +2996,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-21 03:55 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -3036,463 +3008,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>01-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>01200</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>29-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>ESL SHEKOU</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>026D7</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>20-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>01097</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>28-Oct-2026</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>23-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>01069</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>31-Oct-2026</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>11-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>30-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>24-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>01098</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>01-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>27-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>ZHONG YI RUN HAI</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>2642E</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>04-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>28-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>01099</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>05-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>31-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>01071</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>08-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>01-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>01200</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>09-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>2026-10-21 03:55 UTC</t>
+          <t>2026-10-22 03:55 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-23
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>11-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>05-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>22-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>08-Dec-2026</t>
+          <t>09-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>28-Dec-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>15-Jan-2027</t>
+          <t>16-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>28-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>18-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>28-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>22-Jan-2027</t>
+          <t>23-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1630,90 +1630,118 @@
           <t>CNTAO→AEJEA</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>QINGDAO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>25-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>EGLX</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>(No schedule found)</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
+          <t>PHOEBE</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>026E7</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>15-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>06083</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1723,12 +1751,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1738,138 +1766,138 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>28-Nov-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1879,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1894,7 +1922,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1904,76 +1932,76 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNTAO→AEJEA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>26-Dec-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1988,7 +2016,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1998,17 +2026,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>18-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2053,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>22-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2035,12 +2063,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>DINGSHENG7</t>
+          <t>CHANGHENG26</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>06068</t>
+          <t>06083</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2050,7 +2078,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2060,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2072,47 +2100,47 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2139,32 +2167,32 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>00443</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2176,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
+          <t>08-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>EGLX</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ESL NINGBO</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>02645</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>30-Nov-2026</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>ESL KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>02648</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>20-Dec-2026</t>
-        </is>
-      </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2233,7 +2261,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2243,32 +2271,32 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>HUAXIN968</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>00646</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2280,12 +2308,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2295,12 +2323,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2310,17 +2338,17 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2337,7 +2365,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2347,12 +2375,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>DINGSHENG7</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>06068</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2362,17 +2390,17 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2384,47 +2412,47 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>CHANGHENG26</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>06085</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2451,12 +2479,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>01207</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2466,17 +2494,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2488,168 +2516,168 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-22 03:54 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2664,183 +2692,183 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>28-Dec-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>18-Jan-2027</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>01207</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2857,34 +2885,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
+          <t>19-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>01068</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
           <t>27-Oct-2026</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>ZHONG YI RUN HAI</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>2642E</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>04-Nov-2026</t>
-        </is>
-      </c>
       <c r="I48" t="inlineStr">
         <is>
           <t>9</t>
@@ -2892,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2904,47 +2932,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>01099</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:59 UTC</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2989,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2976,7 +3004,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>01071</t>
+          <t>01097</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2986,7 +3014,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2996,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-22 03:55 UTC</t>
+          <t>2026-10-23 03:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3013,42 +3041,354 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>01069</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>12-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ECMX</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>KMTC LONG BEACH</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>02644</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>01-Dec-2026</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>24-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>01098</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
           <t>01-Nov-2026</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
         <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ZHONG YI RUN HAI</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2642E</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>04-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>28-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>FEEDER</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>01099</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>05-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>01071</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>08-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>01-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
         <is>
           <t>01200</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>09-Nov-2026</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>2026-10-22 03:55 UTC</t>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-10-23 03:59 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-24
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>11-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -555,12 +555,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>19-Nov-2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -669,22 +669,22 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -701,42 +701,42 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -753,22 +753,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -778,17 +778,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -825,22 +825,22 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -857,42 +857,42 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>05-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -909,22 +909,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -981,22 +981,22 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,42 +1013,42 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>09-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,22 +1065,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>09-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1137,22 +1137,22 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1169,42 +1169,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>25-Dec-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1221,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1293,22 +1293,22 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14-Dec-2026</t>
+          <t>17-Dec-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1335,32 +1335,32 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>06-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1397,22 +1397,22 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>11-Jan-2027</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>17-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,32 +1439,32 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>11-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,42 +1481,42 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>28-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>16-Jan-2027</t>
+          <t>22-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1538,17 +1538,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>18-Jan-2027</t>
+          <t>16-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>28-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1595,32 +1595,32 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>23-Jan-2027</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>28-Nov-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,17 +1818,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>28-Nov-2026</t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>12-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,17 +1922,17 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>26-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>18-Jan-2027</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2167,32 +2167,32 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>00645</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>23-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>00443</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>08-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>02645</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2256,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>HUAXIN968</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>00646</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>DINGSHENG7</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>06068</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2360,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>DINGSHENG7</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>06068</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2427,12 +2427,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>06085</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>06-Nov-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>02-Nov-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2516,37 +2516,37 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,47 +2568,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2635,32 +2635,32 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2672,47 +2672,47 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2724,47 +2724,47 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>28-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>01207</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>18-Jan-2027</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2776,47 +2776,47 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01207</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2828,99 +2828,99 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>01208</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-23 03:58 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>19-Oct-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>01068</t>
+          <t>02702</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>07-Feb-2027</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2932,47 +2932,47 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>20-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>01097</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>29-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>ESL SHEKOU</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>026D7</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2984,47 +2984,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,59 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-10-23 03:59 UTC</t>
+          <t>2026-10-24 03:53 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>04-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>01072</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>12-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-10-24 03:53 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-25
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -555,12 +555,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -575,12 +575,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -627,12 +627,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -669,22 +669,22 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -701,42 +701,42 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -753,22 +753,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -778,17 +778,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -825,22 +825,22 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -857,42 +857,42 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -909,22 +909,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -934,17 +934,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -981,22 +981,22 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,42 +1013,42 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>09-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,22 +1065,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1137,22 +1137,22 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>25-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1169,42 +1169,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,22 +1221,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>10-Dec-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1283,32 +1283,32 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1350,17 +1350,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1387,12 +1387,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1402,17 +1402,17 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>11-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>17-Dec-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>17-Dec-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1506,17 +1506,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>22-Jan-2027</t>
+          <t>11-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,42 +1533,42 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>28-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>16-Jan-2027</t>
+          <t>22-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,22 +1585,22 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>28-Dec-2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1610,17 +1610,17 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>16-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1766,17 +1766,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>28-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,17 +1818,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>12-Dec-2026</t>
+          <t>05-Dec-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>25-Dec-2026</t>
+          <t>12-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-24 03:52 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2135,12 +2135,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>30-Nov-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>20-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>07-Feb-2027</t>
+          <t>14-Feb-2027</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>01097</t>
+          <t>01069</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2999,12 +2999,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3014,17 +3014,17 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>01098</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3088,47 +3088,47 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>27-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ZHONG YI RUN HAI</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2642E</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>12-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>01099</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3207,12 +3207,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ZHONG YI RUN HAI</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2642E</t>
+          <t>01071</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3249,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3264,7 +3264,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>01099</t>
+          <t>01200</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>01071</t>
+          <t>01072</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>01200</t>
+          <t>01201</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3400,47 +3400,47 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>02-Dec-2026</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>01072</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-10-24 03:53 UTC</t>
+          <t>2026-10-25 03:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-26
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -778,17 +778,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>14-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1303,12 +1303,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1506,17 +1506,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>11-Jan-2027</t>
+          <t>12-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:55 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-25 03:51 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-10-25 03:52 UTC</t>
+          <t>2026-10-26 03:56 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-27
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -679,12 +679,12 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -726,17 +726,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>28-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>16-Jan-2027</t>
+          <t>20-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1719,12 +1719,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>12-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1979,12 +1979,12 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-26 03:55 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>22-Oct-2026</t>
+          <t>23-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>06083</t>
+          <t>00645</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>26-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2167,32 +2167,32 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>00443</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2256,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>DINGSHENG7</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>06068</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>DINGSHENG7</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>06068</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2360,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>CHANGHENG26</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>00648</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:17 UTC</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3388,59 +3388,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-10-26 03:56 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>02-Dec-2026</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>ESL BUSAN</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>02649</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>22-Dec-2026</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>2026-10-26 03:56 UTC</t>
+          <t>2026-10-27 04:18 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-28
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,22 +493,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -555,32 +555,32 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>28</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -602,37 +602,37 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>19-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -659,32 +659,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>17-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -721,22 +721,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -753,42 +753,42 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -805,22 +805,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -830,17 +830,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -877,22 +877,22 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -909,27 +909,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -939,12 +939,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1117,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>16-Dec-2026</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>16</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1169,42 +1169,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,22 +1221,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10-Dec-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>25-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>14-Dec-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1283,32 +1283,32 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1553,22 +1553,22 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>22-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:46 UTC</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1662,17 +1662,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>17-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1766,17 +1766,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>05-Dec-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,17 +1818,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>05-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1974,17 +1974,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2063,12 +2063,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>DINGSHENG7</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00645</t>
+          <t>06068</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>30-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2130,17 +2130,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2167,32 +2167,32 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00443</t>
+          <t>00647</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>03-Nov-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>01205</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>23-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2256,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>DINGSHENG7</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>06068</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>00445</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2360,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CHANGHENG26</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>00648</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>02-Nov-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2427,12 +2427,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>06-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2464,47 +2464,47 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2516,37 +2516,37 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>01207</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,47 +2568,47 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>01208</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2687,12 +2687,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02702</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>14-Feb-2027</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>19-Dec-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01207</t>
+          <t>01209</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>08-Jan-2027</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2764,163 +2764,163 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>01098</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>01208</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ZHONG YI RUN HAI</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>02702</t>
+          <t>2642E</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>14-Feb-2027</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-27 04:17 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>23-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>01069</t>
+          <t>01099</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-27 04:18 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -2984,47 +2984,47 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>31-Oct-2026</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>01071</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>15-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>KMTC LONG BEACH</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>02644</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-27 04:18 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>01200</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-27 04:18 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3103,12 +3103,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>ZHONG YI RUN HAI</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2642E</t>
+          <t>01072</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-27 04:18 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>01099</t>
+          <t>01201</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-27 04:18 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>01071</t>
+          <t>01073</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-27 04:18 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>
@@ -3244,151 +3244,47 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>01200</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>16-Dec-2026</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-27 04:18 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>04-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>01072</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>12-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>2026-10-27 04:18 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>05-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>01201</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>13-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>2026-10-27 04:18 UTC</t>
+          <t>2026-10-28 04:47 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-29
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,22 +493,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02642</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -518,17 +518,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>17-Nov-2026</t>
+          <t>13-Nov-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -555,32 +555,32 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>20-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL SHEKOU</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>02642</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -622,17 +622,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>24-Nov-2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>29-Oct-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -659,32 +659,32 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>20-Nov-2026</t>
+          <t>21-Nov-2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -721,22 +721,22 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>17-Nov-2026</t>
+          <t>19-Nov-2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>30-Oct-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -763,32 +763,32 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>24-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -805,32 +805,32 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ESL SHEKOU</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -857,22 +857,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>17-Nov-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -919,32 +919,32 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -981,22 +981,22 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,42 +1013,42 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL WAFA</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02647</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>22-Dec-2026</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,22 +1117,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>01-Dec-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ESL WAFA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02647</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1142,17 +1142,17 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>16-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1169,42 +1169,42 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>22-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>26</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1231,12 +1231,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1246,17 +1246,17 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1283,32 +1283,32 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1345,22 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>07-Jan-2027</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1387,32 +1387,32 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>SOHAR</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>10-Jan-2027</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>17-Dec-2026</t>
+          <t>20-Dec-2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1449,22 +1449,22 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>15-Jan-2027</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>17-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>12-Jan-2027</t>
+          <t>22-Jan-2027</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1533,22 +1533,22 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>01-Jan-2027</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>20-Jan-2027</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1585,42 +1585,42 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>SOHAR</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>20-Jan-2027</t>
+          <t>29-Jan-2027</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>27</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-28 04:46 UTC</t>
+          <t>2026-10-29 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>026E7</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>21-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1766,17 +1766,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>05-Dec-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,17 +1818,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>05-Dec-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>07-Jan-2027</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>25-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1974,17 +1974,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>01-Jan-2027</t>
+          <t>18-Dec-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>10-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>02-Nov-2026</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2130,17 +2130,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>21-Nov-2026</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>02-Nov-2026</t>
+          <t>29-Oct-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2167,22 +2167,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CHANGHENG27</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00647</t>
+          <t>00443</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2204,47 +2204,47 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>03-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>01205</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>23-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2256,47 +2256,47 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>02-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>CHANGHENG27</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>00647</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
           <t>NINGBO</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>07-Dec-2026</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>ESL KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>02648</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,47 +2308,47 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>COSCO FOS</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>00445</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>07-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2360,47 +2360,47 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>XINGANG</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>04-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>00445</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>08-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>ESL NINGBO</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>02645</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>07-Nov-2026</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>07-Dec-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2427,12 +2427,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>CHANGHENG27</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>01206</t>
+          <t>00649</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2442,17 +2442,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>14-Nov-2026</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>02652</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2494,17 +2494,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>17-Jan-2027</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>12-Nov-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2531,32 +2531,32 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>COSCO FOS</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>01207</t>
+          <t>00446</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>31-Dec-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2568,12 +2568,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NINGBO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>03-Dec-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>02653</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2598,17 +2598,17 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>07-Dec-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>01208</t>
+          <t>01206</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>24-Jan-2027</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2687,12 +2687,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>02702</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>14-Feb-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>19-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>01209</t>
+          <t>01207</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>08-Jan-2027</t>
+          <t>31-Dec-2026</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2764,180 +2764,180 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>01098</t>
+          <t>02653</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>15-Nov-2026</t>
+          <t>15-Dec-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>KMTC LONG BEACH</t>
+          <t>FEEDER</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>02644</t>
+          <t>01208</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>04-Dec-2026</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>24-Jan-2027</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>ZHONG YI RUN HAI</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2642E</t>
+          <t>02702</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>14-Feb-2027</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CNWUH→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>19-Dec-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2952,27 +2952,27 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>01099</t>
+          <t>01209</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>NINGBO</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>08-Jan-2027</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2999,12 +2999,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>ZHONG YI RUN HAI</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>01071</t>
+          <t>2642E</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>04-Nov-2026</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3036,47 +3036,47 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>01-Nov-2026</t>
+          <t>15-Nov-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>FEEDER</t>
+          <t>KMTC LONG BEACH</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>01200</t>
+          <t>02644</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>09-Nov-2026</t>
+          <t>04-Dec-2026</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>04-Nov-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>01072</t>
+          <t>01099</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>12-Nov-2026</t>
+          <t>05-Nov-2026</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>05-Nov-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>01201</t>
+          <t>01071</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>13-Nov-2026</t>
+          <t>08-Nov-2026</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>01-Nov-2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>01073</t>
+          <t>01200</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>09-Nov-2026</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-28 04:47 UTC</t>
+          <t>2026-10-29 04:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3244,47 +3244,255 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>04-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>01072</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>30-Nov-2026</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>12-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-10-29 04:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>05-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>01201</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>13-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-10-29 04:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>08-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>01073</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>16-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>2026-10-29 04:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>28-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>ECMX</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>ESL WAFA</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>02647</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>KHOR FAKKAN</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>16-Dec-2026</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>2026-10-28 04:47 UTC</t>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>15-Dec-2026</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>2026-10-29 04:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>CNWUH→AEJEA</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>09-Nov-2026</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>01202</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>17-Nov-2026</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>2026-10-29 04:59 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-30
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -939,12 +939,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -991,12 +991,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>30-Nov-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>16-Dec-2026</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-29 04:57 UTC</t>
+          <t>2026-10-30 04:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>28-Oct-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>026E7</t>
+          <t>02643</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1662,17 +1662,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>17-Nov-2026</t>
+          <t>21-Nov-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>28-Oct-2026</t>
+          <t>10-Nov-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1699,12 +1699,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>02643</t>
+          <t>02645</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1714,17 +1714,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>21-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10-Nov-2026</t>
+          <t>18-Nov-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>02645</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1766,17 +1766,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>29-Nov-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>16-Nov-2026</t>
+          <t>05-Dec-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1803,12 +1803,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ESL LAEM CHABANG</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>02646</t>
+          <t>02648</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1818,17 +1818,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>06-Dec-2026</t>
+          <t>27-Dec-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1845,7 +1845,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>05-Dec-2026</t>
+          <t>11-Dec-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1855,12 +1855,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02650</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1870,17 +1870,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>03-Jan-2027</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>11-Dec-2026</t>
+          <t>13-Dec-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>SSF TINA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>02650</t>
+          <t>02649</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1922,17 +1922,17 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>03-Jan-2027</t>
+          <t>04-Jan-2027</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>13-Dec-2026</t>
+          <t>18-Dec-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>SSF TINA</t>
+          <t>KMTC DOHA</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>02649</t>
+          <t>02651</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1974,17 +1974,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>04-Jan-2027</t>
+          <t>10-Jan-2027</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>18-Dec-2026</t>
+          <t>25-Dec-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2011,12 +2011,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>KMTC DOHA</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>02651</t>
+          <t>02652</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>10-Jan-2027</t>
+          <t>17-Jan-2027</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>18-Nov-2026</t>
+          <t>20-Nov-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2499,12 +2499,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>03-Dec-2026</t>
+          <t>16-Nov-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>ESL LAEM CHABANG</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>02648</t>
+          <t>02646</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2598,17 +2598,17 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>27-Dec-2026</t>
+          <t>06-Dec-2026</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-29 04:58 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3405,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>28-Nov-2026</t>
+          <t>29-Nov-2026</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>15-Dec-2026</t>
+          <t>16-Dec-2026</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-10-29 04:59 UTC</t>
+          <t>2026-10-30 04:58 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-10-31
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-30 04:57 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:44 UTC</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-10-30 04:58 UTC</t>
+          <t>2026-10-31 04:45 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>